<commit_message>
fix: dynamic sheet import
</commit_message>
<xml_diff>
--- a/public/files/IQMY-Alpro eResult Checking List_17Sep-18Sep2025.xlsx
+++ b/public/files/IQMY-Alpro eResult Checking List_17Sep-18Sep2025.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sadrina.fooad\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\blood-stream-v1\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0E4B7B-3499-4DEA-8A47-F85C59EA5435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F7CB3F-BC46-4EE3-B664-FCA3F84BB06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EF9506C3-AC4A-49CD-B1B0-86138CFB1ABB}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{EF9506C3-AC4A-49CD-B1B0-86138CFB1ABB}"/>
   </bookViews>
   <sheets>
     <sheet name="17-18Sep" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,10 +36,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>PREFIX</t>
+    <t>Prefix</t>
   </si>
   <si>
-    <t>NUM</t>
+    <t>Lab Number</t>
   </si>
 </sst>
 </file>
@@ -422,9 +420,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19317F55-D7F9-48BD-8C4E-6661D92378D6}">
   <dimension ref="A1:B47"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,7 +430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>25</v>
       </c>
@@ -440,7 +438,7 @@
         <v>8207989</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>25</v>
       </c>
@@ -448,7 +446,7 @@
         <v>8207997</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>25</v>
       </c>
@@ -456,7 +454,7 @@
         <v>8792143</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>25</v>
       </c>
@@ -464,7 +462,7 @@
         <v>1999169</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>25</v>
       </c>
@@ -472,7 +470,7 @@
         <v>1999313</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>25</v>
       </c>
@@ -480,7 +478,7 @@
         <v>1999322</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>25</v>
       </c>
@@ -488,7 +486,7 @@
         <v>1999340</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>25</v>
       </c>
@@ -496,7 +494,7 @@
         <v>1999130</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>25</v>
       </c>
@@ -504,7 +502,7 @@
         <v>1999131</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>25</v>
       </c>
@@ -512,7 +510,7 @@
         <v>1999132</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>25</v>
       </c>
@@ -520,7 +518,7 @@
         <v>1999145</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>25</v>
       </c>
@@ -528,7 +526,7 @@
         <v>1999135</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>25</v>
       </c>
@@ -536,7 +534,7 @@
         <v>1999178</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>25</v>
       </c>
@@ -544,7 +542,7 @@
         <v>1999170</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>25</v>
       </c>
@@ -552,7 +550,7 @@
         <v>1999170</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>25</v>
       </c>
@@ -560,7 +558,7 @@
         <v>1999180</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>25</v>
       </c>
@@ -568,7 +566,7 @@
         <v>1999188</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>25</v>
       </c>
@@ -576,7 +574,7 @@
         <v>1939827</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>25</v>
       </c>
@@ -584,7 +582,7 @@
         <v>1939826</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>25</v>
       </c>
@@ -592,7 +590,7 @@
         <v>1939832</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>25</v>
       </c>
@@ -600,7 +598,7 @@
         <v>1939828</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>25</v>
       </c>
@@ -608,7 +606,7 @@
         <v>1939829</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>25</v>
       </c>
@@ -616,7 +614,7 @@
         <v>2021070</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>25</v>
       </c>
@@ -624,7 +622,7 @@
         <v>2021072</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -632,7 +630,7 @@
         <v>2021073</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -640,7 +638,7 @@
         <v>1999259</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>25</v>
       </c>
@@ -648,7 +646,7 @@
         <v>1999258</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>25</v>
       </c>
@@ -656,7 +654,7 @@
         <v>2021074</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>25</v>
       </c>
@@ -664,7 +662,7 @@
         <v>2143476</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>25</v>
       </c>
@@ -672,7 +670,7 @@
         <v>2143477</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>25</v>
       </c>
@@ -680,7 +678,7 @@
         <v>1999284</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>25</v>
       </c>
@@ -688,7 +686,7 @@
         <v>1999280</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>25</v>
       </c>
@@ -696,7 +694,7 @@
         <v>1914385</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>25</v>
       </c>
@@ -704,7 +702,7 @@
         <v>1433515</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>25</v>
       </c>
@@ -712,7 +710,7 @@
         <v>1433514</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>25</v>
       </c>
@@ -720,7 +718,7 @@
         <v>1999341</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>25</v>
       </c>
@@ -728,7 +726,7 @@
         <v>2148676</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>25</v>
       </c>
@@ -736,7 +734,7 @@
         <v>2021146</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>25</v>
       </c>
@@ -744,7 +742,7 @@
         <v>1898533</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>25</v>
       </c>
@@ -752,7 +750,7 @@
         <v>1999362</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>25</v>
       </c>
@@ -760,7 +758,7 @@
         <v>1999362</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>25</v>
       </c>
@@ -768,7 +766,7 @@
         <v>1784577</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>25</v>
       </c>
@@ -776,7 +774,7 @@
         <v>1939860</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>25</v>
       </c>
@@ -784,7 +782,7 @@
         <v>1888005</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>25</v>
       </c>
@@ -792,7 +790,7 @@
         <v>1888002</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>25</v>
       </c>

</xml_diff>